<commit_message>
docs: refresh official xlsx deliverables (R005_2 routing, R-BOM-001 severity, endpoint 2.0m); keep spot-check data local-only
</commit_message>
<xml_diff>
--- a/docs/官方可自动执行规则清单.xlsx
+++ b/docs/官方可自动执行规则清单.xlsx
@@ -481,11 +481,11 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>R001(文件完整性)、R002(图层完整性)、R003(图层命名)、R004(几何类型)、R005(必填字段非空)、R005_1(PM↔ZPM双向)、R005_3(光缆↔PM)、R005_4(端点孤立)、R007(编码唯一)、R008(引用存在)、R009(孤立设备)、R010(端点重合)、R011(容量超限)、R013(设备覆盖)、R014(光缆交越)、R015(间距)、R016(空图层)、R017(坐标系4490)、R018(字段类型)、R019(PM端口容量)、R020(PBO容量)、R021(必填字段存在)、R022(PBO覆盖)、R023(端点断裂)、R027(PM在ZPM内)、R028(PBO在ZPM内)、R032(字段长度)、R033(官方图层非空)、R-BOM-001(BOM物料匹配)、R-FIBER-001(纤芯表重复)、R-FIBER-002(同路由占用推断)</t>
+          <t>R001(文件完整性)、R002(图层完整性)、R003(图层命名)、R004(几何类型)、R005(必填字段非空)、R005_1(PM↔ZPM双向)、R005_2(PBO↔PM主从)、R005_3(光缆↔PM)、R005_4(端点孤立)、R007(编码唯一)、R008(引用存在)、R009(孤立设备)、R010(端点重合)、R011(容量超限)、R013(设备覆盖)、R014(光缆交越)、R015(间距)、R016(空图层)、R017(坐标系4490)、R018(字段类型)、R019(PM端口容量)、R020(PBO容量)、R021(必填字段存在)、R022(PBO覆盖)、R023(端点断裂)、R027(PM在ZPM内)、R028(PBO在ZPM内)、R032(字段长度)、R033(官方图层非空)、R-BOM-001(BOM物料匹配)、R-FIBER-001(纤芯表重复)、R-FIBER-002(同路由占用推断)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -521,11 +521,11 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>R001(文件完整性)、R002(图层完整性)、R003(图层命名)、R004(几何类型)、R005(必填字段非空)、R005_1(PM↔ZPM双向)、R005_3(光缆↔PM)、R005_4(端点孤立)、R007(编码唯一)、R008(引用存在)、R009(孤立设备)、R010(端点重合)、R011(容量超限)、R013(设备覆盖)、R014(光缆交越)、R015(间距)、R016(空图层)、R017(坐标系4490)、R018(字段类型)、R019(PM端口容量)、R020(PBO容量)、R021(必填字段存在)、R022(PBO覆盖)、R023(端点断裂)、R027(PM在ZPM内)、R028(PBO在ZPM内)、R032(字段长度)、R033(官方图层非空)、R-BOM-001(BOM物料匹配)、R-FIBER-001(纤芯表重复)、R-FIBER-002(同路由占用推断)</t>
+          <t>R001(文件完整性)、R002(图层完整性)、R003(图层命名)、R004(几何类型)、R005(必填字段非空)、R005_1(PM↔ZPM双向)、R005_2(PBO↔PM主从)、R005_3(光缆↔PM)、R005_4(端点孤立)、R007(编码唯一)、R008(引用存在)、R009(孤立设备)、R010(端点重合)、R011(容量超限)、R013(设备覆盖)、R014(光缆交越)、R015(间距)、R016(空图层)、R017(坐标系4490)、R018(字段类型)、R019(PM端口容量)、R020(PBO容量)、R021(必填字段存在)、R022(PBO覆盖)、R023(端点断裂)、R027(PM在ZPM内)、R028(PBO在ZPM内)、R032(字段长度)、R033(官方图层非空)、R-BOM-001(BOM物料匹配)、R-FIBER-001(纤芯表重复)、R-FIBER-002(同路由占用推断)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -541,11 +541,11 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>R001(文件完整性)、R002(图层完整性)、R003(图层命名)、R004(几何类型)、R005(必填字段非空)、R005_1(PM↔ZPM双向)、R005_3(光缆↔PM)、R005_4(端点孤立)、R007(编码唯一)、R008(引用存在)、R009(孤立设备)、R010(端点重合)、R011(容量超限)、R013(设备覆盖)、R014(光缆交越)、R015(间距)、R016(空图层)、R017(坐标系4490)、R018(字段类型)、R019(PM端口容量)、R020(PBO容量)、R021(必填字段存在)、R022(PBO覆盖)、R023(端点断裂)、R027(PM在ZPM内)、R028(PBO在ZPM内)、R032(字段长度)、R033(官方图层非空)、R-BOM-001(BOM物料匹配)、R-FIBER-001(纤芯表重复)、R-FIBER-002(同路由占用推断)</t>
+          <t>R001(文件完整性)、R002(图层完整性)、R003(图层命名)、R004(几何类型)、R005(必填字段非空)、R005_1(PM↔ZPM双向)、R005_2(PBO↔PM主从)、R005_3(光缆↔PM)、R005_4(端点孤立)、R007(编码唯一)、R008(引用存在)、R009(孤立设备)、R010(端点重合)、R011(容量超限)、R013(设备覆盖)、R014(光缆交越)、R015(间距)、R016(空图层)、R017(坐标系4490)、R018(字段类型)、R019(PM端口容量)、R020(PBO容量)、R021(必填字段存在)、R022(PBO覆盖)、R023(端点断裂)、R027(PM在ZPM内)、R028(PBO在ZPM内)、R032(字段长度)、R033(官方图层非空)、R-BOM-001(BOM物料匹配)、R-FIBER-001(纤芯表重复)、R-FIBER-002(同路由占用推断)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -561,11 +561,11 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>R001(文件完整性)、R002(图层完整性)、R003(图层命名)、R004(几何类型)、R005(必填字段非空)、R005_1(PM↔ZPM双向)、R005_3(光缆↔PM)、R005_4(端点孤立)、R007(编码唯一)、R008(引用存在)、R009(孤立设备)、R010(端点重合)、R011(容量超限)、R013(设备覆盖)、R014(光缆交越)、R015(间距)、R016(空图层)、R017(坐标系4490)、R018(字段类型)、R019(PM端口容量)、R020(PBO容量)、R021(必填字段存在)、R022(PBO覆盖)、R023(端点断裂)、R027(PM在ZPM内)、R028(PBO在ZPM内)、R032(字段长度)、R033(官方图层非空)、R-BOM-001(BOM物料匹配)、R-FIBER-001(纤芯表重复)、R-FIBER-002(同路由占用推断)</t>
+          <t>R001(文件完整性)、R002(图层完整性)、R003(图层命名)、R004(几何类型)、R005(必填字段非空)、R005_1(PM↔ZPM双向)、R005_2(PBO↔PM主从)、R005_3(光缆↔PM)、R005_4(端点孤立)、R007(编码唯一)、R008(引用存在)、R009(孤立设备)、R010(端点重合)、R011(容量超限)、R013(设备覆盖)、R014(光缆交越)、R015(间距)、R016(空图层)、R017(坐标系4490)、R018(字段类型)、R019(PM端口容量)、R020(PBO容量)、R021(必填字段存在)、R022(PBO覆盖)、R023(端点断裂)、R027(PM在ZPM内)、R028(PBO在ZPM内)、R032(字段长度)、R033(官方图层非空)、R-BOM-001(BOM物料匹配)、R-FIBER-001(纤芯表重复)、R-FIBER-002(同路由占用推断)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">

</xml_diff>